<commit_message>
style(ui): update shared UI primitives, navigation, and brand palette
- Refine shared UI components: Badge, Button, Card, Navbar, and PageHeader.
- Add subtle brand typography, gradients, and shadow utilities.
- Add spreadsheet snapshot for joined export testing.
</commit_message>
<xml_diff>
--- a/visualisasi-capaian-indikator-kesehatan.xlsx
+++ b/visualisasi-capaian-indikator-kesehatan.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -54,8 +54,20 @@
       <b/>
       <color rgb="FFFFFF"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <b/>
+      <color rgb="3730A3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <b/>
+      <color rgb="3730A3"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -78,8 +90,20 @@
         <bgColor/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF2FF"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF2FF"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -94,11 +118,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="C7D2FE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="C7D2FE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="C7D2FE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="C7D2FE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -106,6 +152,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -439,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -550,9 +602,26 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="5" t="str">
+        <v>Target</v>
+      </c>
+      <c r="B7" s="6" t="str">
+        <v>-</v>
+      </c>
+      <c r="C7" s="6" t="str">
+        <v>-</v>
+      </c>
+      <c r="D7" s="6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E7" s="6" t="str">
+        <v>-</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>